<commit_message>
General Flow Tikz Diagram update
</commit_message>
<xml_diff>
--- a/ProjectManagement/EvaluationHWAndProject.xlsx
+++ b/ProjectManagement/EvaluationHWAndProject.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\gthub\ML26-03-Car-Licence-Plate-Identification-with-a-Jetson-Nano\ProjectManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39945EBF-606D-4BF5-A2DB-67107DFF197C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A84961D-D91D-4C59-A025-85C8B66A1D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1802,6 +1802,33 @@
       <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1828,33 +1855,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2142,16 +2142,16 @@
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.21875" customWidth="1"/>
     <col min="3" max="3" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.21875" style="38" customWidth="1"/>
+    <col min="4" max="4" width="39.21875" style="29" customWidth="1"/>
     <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:6" ht="33.6" x14ac:dyDescent="0.65">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="38" t="s">
         <v>392</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -2159,11 +2159,11 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="39" t="s">
         <v>393</v>
       </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -2185,7 +2185,7 @@
       <c r="C10" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="30" t="s">
         <v>87</v>
       </c>
       <c r="F10" t="s">
@@ -2202,7 +2202,7 @@
       <c r="C11" s="3">
         <v>7026787</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="29" t="s">
         <v>400</v>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
         <v>166</v>
       </c>
       <c r="C28" s="13"/>
-      <c r="D28" s="40"/>
+      <c r="D28" s="31"/>
       <c r="E28" s="13">
         <v>-25</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>166</v>
       </c>
       <c r="C30" s="12"/>
-      <c r="D30" s="41"/>
+      <c r="D30" s="32"/>
       <c r="E30" s="12">
         <v>-25</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>167</v>
       </c>
       <c r="C31" s="12"/>
-      <c r="D31" s="41"/>
+      <c r="D31" s="32"/>
       <c r="E31" s="12">
         <v>-25</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>167</v>
       </c>
       <c r="C33" s="13"/>
-      <c r="D33" s="40"/>
+      <c r="D33" s="31"/>
       <c r="E33" s="13">
         <v>-25</v>
       </c>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
-      <c r="D36" s="40"/>
+      <c r="D36" s="31"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
     </row>
@@ -2393,7 +2393,7 @@
         <v>3</v>
       </c>
       <c r="C37" s="13"/>
-      <c r="D37" s="40"/>
+      <c r="D37" s="31"/>
       <c r="E37" s="13"/>
       <c r="F37" s="13">
         <v>10</v>
@@ -2405,7 +2405,7 @@
         <v>28</v>
       </c>
       <c r="C38" s="13"/>
-      <c r="D38" s="40"/>
+      <c r="D38" s="31"/>
       <c r="E38" s="13"/>
       <c r="F38" s="13">
         <v>10</v>
@@ -2417,7 +2417,7 @@
         <v>4</v>
       </c>
       <c r="C39" s="13"/>
-      <c r="D39" s="40"/>
+      <c r="D39" s="31"/>
       <c r="E39" s="13"/>
       <c r="F39" s="13">
         <v>10</v>
@@ -2429,7 +2429,7 @@
         <v>5</v>
       </c>
       <c r="C40" s="13"/>
-      <c r="D40" s="40"/>
+      <c r="D40" s="31"/>
       <c r="E40" s="13"/>
       <c r="F40" s="13">
         <v>10</v>
@@ -2441,7 +2441,7 @@
         <v>6</v>
       </c>
       <c r="C41" s="13"/>
-      <c r="D41" s="40"/>
+      <c r="D41" s="31"/>
       <c r="E41" s="13"/>
       <c r="F41" s="13">
         <v>10</v>
@@ -2453,7 +2453,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="13"/>
-      <c r="D42" s="40"/>
+      <c r="D42" s="31"/>
       <c r="E42" s="13"/>
       <c r="F42" s="13">
         <v>10</v>
@@ -2463,7 +2463,7 @@
       <c r="A43" s="15"/>
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
-      <c r="D43" s="40"/>
+      <c r="D43" s="31"/>
       <c r="E43" s="13"/>
       <c r="F43" s="13"/>
     </row>
@@ -2475,7 +2475,7 @@
       <c r="C44" s="13" t="s">
         <v>257</v>
       </c>
-      <c r="D44" s="40"/>
+      <c r="D44" s="31"/>
       <c r="E44" s="13"/>
       <c r="F44" s="13">
         <v>4</v>
@@ -2487,7 +2487,7 @@
       <c r="C45" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="D45" s="40"/>
+      <c r="D45" s="31"/>
       <c r="E45" s="13"/>
       <c r="F45" s="13">
         <v>6</v>
@@ -2499,7 +2499,7 @@
       <c r="C46" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="D46" s="40"/>
+      <c r="D46" s="31"/>
       <c r="E46" s="13"/>
       <c r="F46" s="13">
         <v>10</v>
@@ -2511,7 +2511,7 @@
       <c r="C47" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="D47" s="40"/>
+      <c r="D47" s="31"/>
       <c r="E47" s="13"/>
       <c r="F47" s="13">
         <v>5</v>
@@ -2523,7 +2523,7 @@
       <c r="C48" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="D48" s="40"/>
+      <c r="D48" s="31"/>
       <c r="E48" s="13"/>
       <c r="F48" s="13">
         <v>5</v>
@@ -2535,7 +2535,7 @@
       <c r="C49" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="D49" s="40"/>
+      <c r="D49" s="31"/>
       <c r="E49" s="13"/>
       <c r="F49" s="13">
         <v>5</v>
@@ -2547,7 +2547,7 @@
       <c r="C50" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="D50" s="40"/>
+      <c r="D50" s="31"/>
       <c r="E50" s="13"/>
       <c r="F50" s="13">
         <v>5</v>
@@ -2557,7 +2557,7 @@
       <c r="A51" s="13"/>
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
-      <c r="D51" s="42" t="s">
+      <c r="D51" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E51" s="28">
@@ -2579,7 +2579,7 @@
       <c r="A54" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="D54" s="43"/>
+      <c r="D54" s="34"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="16" t="s">
@@ -2594,7 +2594,7 @@
       <c r="F55" s="14">
         <v>10</v>
       </c>
-      <c r="G55" s="31" t="s">
+      <c r="G55" s="40" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       <c r="F56" s="14">
         <v>5</v>
       </c>
-      <c r="G56" s="31"/>
+      <c r="G56" s="40"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="16"/>
@@ -2622,7 +2622,7 @@
       <c r="F57" s="14">
         <v>5</v>
       </c>
-      <c r="G57" s="31"/>
+      <c r="G57" s="40"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="16"/>
@@ -2635,7 +2635,7 @@
       <c r="F58" s="14">
         <v>5</v>
       </c>
-      <c r="G58" s="31"/>
+      <c r="G58" s="40"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="16"/>
@@ -2648,7 +2648,7 @@
       <c r="F59" s="14">
         <v>10</v>
       </c>
-      <c r="G59" s="31"/>
+      <c r="G59" s="40"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="16"/>
@@ -2661,7 +2661,7 @@
       <c r="F60" s="14">
         <v>5</v>
       </c>
-      <c r="G60" s="31"/>
+      <c r="G60" s="40"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="16"/>
@@ -2674,7 +2674,7 @@
       <c r="F61" s="14">
         <v>10</v>
       </c>
-      <c r="G61" s="31"/>
+      <c r="G61" s="40"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="16"/>
@@ -2687,7 +2687,7 @@
       <c r="F62" s="14">
         <v>5</v>
       </c>
-      <c r="G62" s="31"/>
+      <c r="G62" s="40"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="16"/>
@@ -2700,7 +2700,7 @@
       <c r="F63" s="14">
         <v>5</v>
       </c>
-      <c r="G63" s="31"/>
+      <c r="G63" s="40"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" s="16"/>
@@ -2713,7 +2713,7 @@
       <c r="F64" s="14">
         <v>5</v>
       </c>
-      <c r="G64" s="31"/>
+      <c r="G64" s="40"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" s="16"/>
@@ -2726,7 +2726,7 @@
       <c r="F65" s="14">
         <v>5</v>
       </c>
-      <c r="G65" s="31"/>
+      <c r="G65" s="40"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" s="16"/>
@@ -2739,7 +2739,7 @@
       <c r="F66" s="14">
         <v>5</v>
       </c>
-      <c r="G66" s="31"/>
+      <c r="G66" s="40"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" s="16"/>
@@ -2752,20 +2752,20 @@
       <c r="F67" s="14">
         <v>5</v>
       </c>
-      <c r="G67" s="31"/>
+      <c r="G67" s="40"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" s="16"/>
       <c r="B68" s="14"/>
       <c r="C68" s="14"/>
-      <c r="D68" s="42" t="s">
+      <c r="D68" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E68" s="28">
         <v>1</v>
       </c>
       <c r="F68" s="14"/>
-      <c r="G68" s="31"/>
+      <c r="G68" s="40"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
@@ -2782,7 +2782,7 @@
       <c r="A70" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="D70" s="43"/>
+      <c r="D70" s="34"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" s="16" t="s">
@@ -2797,7 +2797,7 @@
       <c r="F71" s="14">
         <v>10</v>
       </c>
-      <c r="G71" s="34" t="s">
+      <c r="G71" s="43" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2812,7 +2812,7 @@
       <c r="F72" s="14">
         <v>5</v>
       </c>
-      <c r="G72" s="34"/>
+      <c r="G72" s="43"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="16"/>
@@ -2825,7 +2825,7 @@
       <c r="F73" s="14">
         <v>5</v>
       </c>
-      <c r="G73" s="34"/>
+      <c r="G73" s="43"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="16"/>
@@ -2838,7 +2838,7 @@
       <c r="F74" s="14">
         <v>5</v>
       </c>
-      <c r="G74" s="34"/>
+      <c r="G74" s="43"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="16"/>
@@ -2851,7 +2851,7 @@
       <c r="F75" s="14">
         <v>10</v>
       </c>
-      <c r="G75" s="34"/>
+      <c r="G75" s="43"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="16"/>
@@ -2864,20 +2864,20 @@
       <c r="F76" s="14">
         <v>5</v>
       </c>
-      <c r="G76" s="34"/>
+      <c r="G76" s="43"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="16"/>
       <c r="B77" s="14"/>
       <c r="C77" s="14"/>
-      <c r="D77" s="42" t="s">
+      <c r="D77" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E77" s="28">
         <v>1</v>
       </c>
       <c r="F77" s="14"/>
-      <c r="G77" s="34"/>
+      <c r="G77" s="43"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="1"/>
@@ -2908,12 +2908,12 @@
       <c r="C81" s="8" t="s">
         <v>316</v>
       </c>
-      <c r="D81" s="44"/>
+      <c r="D81" s="35"/>
       <c r="E81" s="8"/>
       <c r="F81" s="8">
         <v>0</v>
       </c>
-      <c r="G81" s="35" t="s">
+      <c r="G81" s="44" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2925,12 +2925,12 @@
       <c r="C82" s="8" t="s">
         <v>383</v>
       </c>
-      <c r="D82" s="44"/>
+      <c r="D82" s="35"/>
       <c r="E82" s="8"/>
       <c r="F82" s="8">
         <v>30</v>
       </c>
-      <c r="G82" s="35"/>
+      <c r="G82" s="44"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="7"/>
@@ -2938,12 +2938,12 @@
       <c r="C83" s="8" t="s">
         <v>384</v>
       </c>
-      <c r="D83" s="44"/>
+      <c r="D83" s="35"/>
       <c r="E83" s="8"/>
       <c r="F83" s="8">
         <v>10</v>
       </c>
-      <c r="G83" s="35"/>
+      <c r="G83" s="44"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="7"/>
@@ -2951,25 +2951,25 @@
       <c r="C84" s="8" t="s">
         <v>385</v>
       </c>
-      <c r="D84" s="44"/>
+      <c r="D84" s="35"/>
       <c r="E84" s="8"/>
       <c r="F84" s="8">
         <v>10</v>
       </c>
-      <c r="G84" s="35"/>
+      <c r="G84" s="44"/>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="7"/>
       <c r="B85" s="7"/>
       <c r="C85" s="7"/>
-      <c r="D85" s="42" t="s">
+      <c r="D85" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E85" s="28">
         <v>1</v>
       </c>
       <c r="F85" s="7"/>
-      <c r="G85" s="35"/>
+      <c r="G85" s="44"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="1"/>
@@ -2999,7 +2999,7 @@
         <v>316</v>
       </c>
       <c r="C89" s="13"/>
-      <c r="D89" s="40"/>
+      <c r="D89" s="31"/>
       <c r="E89" s="13"/>
       <c r="F89" s="13">
         <v>10</v>
@@ -3011,7 +3011,7 @@
         <v>131</v>
       </c>
       <c r="C90" s="13"/>
-      <c r="D90" s="40"/>
+      <c r="D90" s="31"/>
       <c r="E90" s="13"/>
       <c r="F90" s="13">
         <v>5</v>
@@ -3023,7 +3023,7 @@
         <v>235</v>
       </c>
       <c r="C91" s="13"/>
-      <c r="D91" s="40"/>
+      <c r="D91" s="31"/>
       <c r="E91" s="13"/>
       <c r="F91" s="13">
         <v>5</v>
@@ -3035,7 +3035,7 @@
         <v>8</v>
       </c>
       <c r="C92" s="13"/>
-      <c r="D92" s="40"/>
+      <c r="D92" s="31"/>
       <c r="E92" s="13"/>
       <c r="F92" s="13">
         <v>5</v>
@@ -3047,7 +3047,7 @@
         <v>132</v>
       </c>
       <c r="C93" s="13"/>
-      <c r="D93" s="40"/>
+      <c r="D93" s="31"/>
       <c r="E93" s="13"/>
       <c r="F93" s="13">
         <v>5</v>
@@ -3059,7 +3059,7 @@
         <v>133</v>
       </c>
       <c r="C94" s="13"/>
-      <c r="D94" s="40"/>
+      <c r="D94" s="31"/>
       <c r="E94" s="13"/>
       <c r="F94" s="13">
         <v>5</v>
@@ -3071,7 +3071,7 @@
         <v>134</v>
       </c>
       <c r="C95" s="13"/>
-      <c r="D95" s="40"/>
+      <c r="D95" s="31"/>
       <c r="E95" s="13"/>
       <c r="F95" s="13">
         <v>5</v>
@@ -3081,7 +3081,7 @@
       <c r="A96" s="15"/>
       <c r="B96" s="13"/>
       <c r="C96" s="13"/>
-      <c r="D96" s="42" t="s">
+      <c r="D96" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E96" s="28">
@@ -3119,7 +3119,7 @@
         <v>8</v>
       </c>
       <c r="C101" s="13"/>
-      <c r="D101" s="40"/>
+      <c r="D101" s="31"/>
       <c r="E101" s="13"/>
       <c r="F101" s="13">
         <v>5</v>
@@ -3131,7 +3131,7 @@
         <v>9</v>
       </c>
       <c r="C102" s="13"/>
-      <c r="D102" s="40"/>
+      <c r="D102" s="31"/>
       <c r="E102" s="13"/>
       <c r="F102" s="13">
         <v>5</v>
@@ -3143,7 +3143,7 @@
         <v>10</v>
       </c>
       <c r="C103" s="13"/>
-      <c r="D103" s="40"/>
+      <c r="D103" s="31"/>
       <c r="E103" s="13"/>
       <c r="F103" s="13">
         <v>5</v>
@@ -3155,7 +3155,7 @@
         <v>11</v>
       </c>
       <c r="C104" s="13"/>
-      <c r="D104" s="40"/>
+      <c r="D104" s="31"/>
       <c r="E104" s="13"/>
       <c r="F104" s="13">
         <v>10</v>
@@ -3167,7 +3167,7 @@
         <v>12</v>
       </c>
       <c r="C105" s="13"/>
-      <c r="D105" s="40"/>
+      <c r="D105" s="31"/>
       <c r="E105" s="13"/>
       <c r="F105" s="13">
         <v>5</v>
@@ -3179,7 +3179,7 @@
         <v>100</v>
       </c>
       <c r="C106" s="13"/>
-      <c r="D106" s="40"/>
+      <c r="D106" s="31"/>
       <c r="E106" s="13"/>
       <c r="F106" s="13">
         <v>5</v>
@@ -3189,7 +3189,7 @@
       <c r="A107" s="13"/>
       <c r="B107" s="13"/>
       <c r="C107" s="13"/>
-      <c r="D107" s="42" t="s">
+      <c r="D107" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E107" s="28">
@@ -3314,7 +3314,7 @@
       <c r="A119" s="14"/>
       <c r="B119" s="24"/>
       <c r="C119" s="14"/>
-      <c r="D119" s="42" t="s">
+      <c r="D119" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E119" s="28">
@@ -3347,14 +3347,14 @@
       <c r="C124" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="D124" s="41"/>
+      <c r="D124" s="32"/>
       <c r="E124" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F124" s="12">
         <v>6</v>
       </c>
-      <c r="G124" s="32" t="s">
+      <c r="G124" s="41" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
       <c r="C125" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="D125" s="41" t="s">
+      <c r="D125" s="32" t="s">
         <v>331</v>
       </c>
       <c r="E125" s="12" t="s">
@@ -3375,13 +3375,13 @@
       <c r="F125" s="12">
         <v>6</v>
       </c>
-      <c r="G125" s="32"/>
+      <c r="G125" s="41"/>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126" s="12"/>
       <c r="B126" s="12"/>
       <c r="C126" s="12"/>
-      <c r="D126" s="41" t="s">
+      <c r="D126" s="32" t="s">
         <v>102</v>
       </c>
       <c r="E126" s="12" t="s">
@@ -3390,7 +3390,7 @@
       <c r="F126" s="12">
         <v>6</v>
       </c>
-      <c r="G126" s="32"/>
+      <c r="G126" s="41"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127" s="12"/>
@@ -3398,14 +3398,14 @@
       <c r="C127" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D127" s="41"/>
+      <c r="D127" s="32"/>
       <c r="E127" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F127" s="12">
         <v>6</v>
       </c>
-      <c r="G127" s="32"/>
+      <c r="G127" s="41"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128" s="12"/>
@@ -3413,14 +3413,14 @@
       <c r="C128" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="D128" s="41"/>
+      <c r="D128" s="32"/>
       <c r="E128" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F128" s="12">
         <v>6</v>
       </c>
-      <c r="G128" s="32"/>
+      <c r="G128" s="41"/>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129" s="12"/>
@@ -3428,27 +3428,27 @@
       <c r="C129" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="D129" s="41"/>
+      <c r="D129" s="32"/>
       <c r="E129" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F129" s="12">
         <v>6</v>
       </c>
-      <c r="G129" s="32"/>
+      <c r="G129" s="41"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130" s="12"/>
       <c r="B130" s="12"/>
       <c r="C130" s="12"/>
-      <c r="D130" s="42" t="s">
+      <c r="D130" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E130" s="28">
         <v>1</v>
       </c>
       <c r="F130" s="12"/>
-      <c r="G130" s="32"/>
+      <c r="G130" s="41"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E131">
@@ -3459,7 +3459,7 @@
         <f>SUM(F124:F129)</f>
         <v>36</v>
       </c>
-      <c r="G131" s="32"/>
+      <c r="G131" s="41"/>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132" s="11" t="s">
@@ -3471,14 +3471,14 @@
       <c r="C132" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="D132" s="41"/>
+      <c r="D132" s="32"/>
       <c r="E132" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F132" s="12">
         <v>10</v>
       </c>
-      <c r="G132" s="32"/>
+      <c r="G132" s="41"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A133" s="12"/>
@@ -3486,7 +3486,7 @@
       <c r="C133" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="D133" s="41" t="s">
+      <c r="D133" s="32" t="s">
         <v>117</v>
       </c>
       <c r="E133" s="12" t="s">
@@ -3495,13 +3495,13 @@
       <c r="F133" s="12">
         <v>5</v>
       </c>
-      <c r="G133" s="32"/>
+      <c r="G133" s="41"/>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A134" s="12"/>
       <c r="B134" s="12"/>
       <c r="C134" s="12"/>
-      <c r="D134" s="41" t="s">
+      <c r="D134" s="32" t="s">
         <v>118</v>
       </c>
       <c r="E134" s="12" t="s">
@@ -3510,13 +3510,13 @@
       <c r="F134" s="12">
         <v>5</v>
       </c>
-      <c r="G134" s="32"/>
+      <c r="G134" s="41"/>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A135" s="11"/>
       <c r="B135" s="12"/>
       <c r="C135" s="12"/>
-      <c r="D135" s="41" t="s">
+      <c r="D135" s="32" t="s">
         <v>103</v>
       </c>
       <c r="E135" s="12" t="s">
@@ -3525,13 +3525,13 @@
       <c r="F135" s="12">
         <v>5</v>
       </c>
-      <c r="G135" s="32"/>
+      <c r="G135" s="41"/>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A136" s="11"/>
       <c r="B136" s="12"/>
       <c r="C136" s="12"/>
-      <c r="D136" s="41" t="s">
+      <c r="D136" s="32" t="s">
         <v>13</v>
       </c>
       <c r="E136" s="12" t="s">
@@ -3540,7 +3540,7 @@
       <c r="F136" s="12">
         <v>5</v>
       </c>
-      <c r="G136" s="32"/>
+      <c r="G136" s="41"/>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A137" s="11"/>
@@ -3548,14 +3548,14 @@
       <c r="C137" s="12" t="s">
         <v>332</v>
       </c>
-      <c r="D137" s="41"/>
+      <c r="D137" s="32"/>
       <c r="E137" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F137" s="12">
         <v>10</v>
       </c>
-      <c r="G137" s="32"/>
+      <c r="G137" s="41"/>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A138" s="12"/>
@@ -3563,14 +3563,14 @@
       <c r="C138" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D138" s="41"/>
+      <c r="D138" s="32"/>
       <c r="E138" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F138" s="12">
         <v>5</v>
       </c>
-      <c r="G138" s="32"/>
+      <c r="G138" s="41"/>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A139" s="12"/>
@@ -3578,27 +3578,27 @@
       <c r="C139" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="D139" s="41"/>
+      <c r="D139" s="32"/>
       <c r="E139" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F139" s="12">
         <v>5</v>
       </c>
-      <c r="G139" s="32"/>
+      <c r="G139" s="41"/>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A140" s="12"/>
       <c r="B140" s="12"/>
       <c r="C140" s="12"/>
-      <c r="D140" s="42" t="s">
+      <c r="D140" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E140" s="28">
         <v>1</v>
       </c>
       <c r="F140" s="12"/>
-      <c r="G140" s="32"/>
+      <c r="G140" s="41"/>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E141">
@@ -3609,7 +3609,7 @@
         <f>SUM(F132:F139)</f>
         <v>50</v>
       </c>
-      <c r="G141" s="32"/>
+      <c r="G141" s="41"/>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A142" s="11" t="s">
@@ -3621,14 +3621,14 @@
       <c r="C142" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="D142" s="41"/>
+      <c r="D142" s="32"/>
       <c r="E142" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F142" s="12">
         <v>6</v>
       </c>
-      <c r="G142" s="32"/>
+      <c r="G142" s="41"/>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A143" s="11" t="s">
@@ -3638,12 +3638,12 @@
       <c r="C143" s="12" t="s">
         <v>336</v>
       </c>
-      <c r="D143" s="41"/>
+      <c r="D143" s="32"/>
       <c r="E143" s="12"/>
       <c r="F143" s="12">
         <v>6</v>
       </c>
-      <c r="G143" s="32"/>
+      <c r="G143" s="41"/>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A144" s="11"/>
@@ -3651,12 +3651,12 @@
       <c r="C144" s="12" t="s">
         <v>337</v>
       </c>
-      <c r="D144" s="41"/>
+      <c r="D144" s="32"/>
       <c r="E144" s="12"/>
       <c r="F144" s="12">
         <v>10</v>
       </c>
-      <c r="G144" s="32"/>
+      <c r="G144" s="41"/>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A145" s="11"/>
@@ -3664,7 +3664,7 @@
       <c r="C145" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="D145" s="41" t="s">
+      <c r="D145" s="32" t="s">
         <v>331</v>
       </c>
       <c r="E145" s="12" t="s">
@@ -3673,13 +3673,13 @@
       <c r="F145" s="12">
         <v>6</v>
       </c>
-      <c r="G145" s="32"/>
+      <c r="G145" s="41"/>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A146" s="12"/>
       <c r="B146" s="12"/>
       <c r="C146" s="12"/>
-      <c r="D146" s="41" t="s">
+      <c r="D146" s="32" t="s">
         <v>102</v>
       </c>
       <c r="E146" s="12" t="s">
@@ -3688,7 +3688,7 @@
       <c r="F146" s="12">
         <v>6</v>
       </c>
-      <c r="G146" s="32"/>
+      <c r="G146" s="41"/>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A147" s="12"/>
@@ -3696,14 +3696,14 @@
       <c r="C147" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D147" s="41"/>
+      <c r="D147" s="32"/>
       <c r="E147" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F147" s="12">
         <v>6</v>
       </c>
-      <c r="G147" s="32"/>
+      <c r="G147" s="41"/>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A148" s="12"/>
@@ -3711,14 +3711,14 @@
       <c r="C148" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="D148" s="41"/>
+      <c r="D148" s="32"/>
       <c r="E148" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F148" s="12">
         <v>6</v>
       </c>
-      <c r="G148" s="32"/>
+      <c r="G148" s="41"/>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A149" s="12"/>
@@ -3726,27 +3726,27 @@
       <c r="C149" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="D149" s="41"/>
+      <c r="D149" s="32"/>
       <c r="E149" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F149" s="12">
         <v>6</v>
       </c>
-      <c r="G149" s="32"/>
+      <c r="G149" s="41"/>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A150" s="12"/>
       <c r="B150" s="12"/>
       <c r="C150" s="12"/>
-      <c r="D150" s="42" t="s">
+      <c r="D150" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E150" s="28">
         <v>1</v>
       </c>
       <c r="F150" s="12"/>
-      <c r="G150" s="32"/>
+      <c r="G150" s="41"/>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E151">
@@ -3757,7 +3757,7 @@
         <f>SUM(F142:F149)</f>
         <v>52</v>
       </c>
-      <c r="G151" s="32"/>
+      <c r="G151" s="41"/>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152" s="11" t="s">
@@ -3769,14 +3769,14 @@
       <c r="C152" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="D152" s="41"/>
+      <c r="D152" s="32"/>
       <c r="E152" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F152" s="12">
         <v>10</v>
       </c>
-      <c r="G152" s="32"/>
+      <c r="G152" s="41"/>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153" s="12"/>
@@ -3784,7 +3784,7 @@
       <c r="C153" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="D153" s="41" t="s">
+      <c r="D153" s="32" t="s">
         <v>117</v>
       </c>
       <c r="E153" s="12" t="s">
@@ -3793,13 +3793,13 @@
       <c r="F153" s="12">
         <v>5</v>
       </c>
-      <c r="G153" s="32"/>
+      <c r="G153" s="41"/>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A154" s="12"/>
       <c r="B154" s="12"/>
       <c r="C154" s="12"/>
-      <c r="D154" s="41" t="s">
+      <c r="D154" s="32" t="s">
         <v>118</v>
       </c>
       <c r="E154" s="12" t="s">
@@ -3808,13 +3808,13 @@
       <c r="F154" s="12">
         <v>5</v>
       </c>
-      <c r="G154" s="32"/>
+      <c r="G154" s="41"/>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A155" s="11"/>
       <c r="B155" s="12"/>
       <c r="C155" s="12"/>
-      <c r="D155" s="41" t="s">
+      <c r="D155" s="32" t="s">
         <v>103</v>
       </c>
       <c r="E155" s="12" t="s">
@@ -3823,13 +3823,13 @@
       <c r="F155" s="12">
         <v>5</v>
       </c>
-      <c r="G155" s="32"/>
+      <c r="G155" s="41"/>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156" s="11"/>
       <c r="B156" s="12"/>
       <c r="C156" s="12"/>
-      <c r="D156" s="41" t="s">
+      <c r="D156" s="32" t="s">
         <v>13</v>
       </c>
       <c r="E156" s="12" t="s">
@@ -3838,7 +3838,7 @@
       <c r="F156" s="12">
         <v>5</v>
       </c>
-      <c r="G156" s="32"/>
+      <c r="G156" s="41"/>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A157" s="11"/>
@@ -3846,12 +3846,12 @@
       <c r="C157" s="12" t="s">
         <v>337</v>
       </c>
-      <c r="D157" s="41"/>
+      <c r="D157" s="32"/>
       <c r="E157" s="12"/>
       <c r="F157" s="12">
         <v>10</v>
       </c>
-      <c r="G157" s="32"/>
+      <c r="G157" s="41"/>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158" s="11"/>
@@ -3859,14 +3859,14 @@
       <c r="C158" s="12" t="s">
         <v>332</v>
       </c>
-      <c r="D158" s="41"/>
+      <c r="D158" s="32"/>
       <c r="E158" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F158" s="12">
         <v>10</v>
       </c>
-      <c r="G158" s="32"/>
+      <c r="G158" s="41"/>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159" s="12"/>
@@ -3874,14 +3874,14 @@
       <c r="C159" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D159" s="41"/>
+      <c r="D159" s="32"/>
       <c r="E159" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F159" s="12">
         <v>5</v>
       </c>
-      <c r="G159" s="32"/>
+      <c r="G159" s="41"/>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160" s="12"/>
@@ -3889,27 +3889,27 @@
       <c r="C160" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="D160" s="41"/>
+      <c r="D160" s="32"/>
       <c r="E160" s="12" t="s">
         <v>319</v>
       </c>
       <c r="F160" s="12">
         <v>5</v>
       </c>
-      <c r="G160" s="32"/>
+      <c r="G160" s="41"/>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161" s="12"/>
       <c r="B161" s="12"/>
       <c r="C161" s="12"/>
-      <c r="D161" s="42" t="s">
+      <c r="D161" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E161" s="28">
         <v>1</v>
       </c>
       <c r="F161" s="12"/>
-      <c r="G161" s="32"/>
+      <c r="G161" s="41"/>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E162">
@@ -3920,7 +3920,7 @@
         <f>SUM(F152:F160)</f>
         <v>60</v>
       </c>
-      <c r="G162" s="32"/>
+      <c r="G162" s="41"/>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G163" s="27"/>
@@ -3969,7 +3969,7 @@
       <c r="A167" s="16"/>
       <c r="B167" s="14"/>
       <c r="C167" s="14"/>
-      <c r="D167" s="42" t="s">
+      <c r="D167" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E167" s="28">
@@ -4056,7 +4056,7 @@
       <c r="A174" s="16"/>
       <c r="B174" s="14"/>
       <c r="C174" s="14"/>
-      <c r="D174" s="42" t="s">
+      <c r="D174" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E174" s="28">
@@ -4219,7 +4219,7 @@
       <c r="A186" s="14"/>
       <c r="B186" s="14"/>
       <c r="C186" s="14"/>
-      <c r="D186" s="42" t="s">
+      <c r="D186" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E186" s="28">
@@ -4371,7 +4371,7 @@
       <c r="A197" s="14"/>
       <c r="B197" s="14"/>
       <c r="C197" s="14"/>
-      <c r="D197" s="42" t="s">
+      <c r="D197" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E197" s="28">
@@ -4431,7 +4431,7 @@
       <c r="A202" s="16"/>
       <c r="B202" s="14"/>
       <c r="C202" s="14"/>
-      <c r="D202" s="42" t="s">
+      <c r="D202" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E202" s="28">
@@ -4457,7 +4457,7 @@
       <c r="A205" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="D205" s="43"/>
+      <c r="D205" s="34"/>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A206" s="1" t="s">
@@ -4469,7 +4469,7 @@
       <c r="C206" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="D206" s="41"/>
+      <c r="D206" s="32"/>
       <c r="E206" s="12"/>
       <c r="F206" s="12">
         <v>5</v>
@@ -4482,7 +4482,7 @@
       <c r="C207" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="D207" s="41"/>
+      <c r="D207" s="32"/>
       <c r="E207" s="12"/>
       <c r="F207" s="12">
         <v>5</v>
@@ -4494,7 +4494,7 @@
       <c r="C208" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="D208" s="41"/>
+      <c r="D208" s="32"/>
       <c r="E208" s="12"/>
       <c r="F208" s="12">
         <v>5</v>
@@ -4506,7 +4506,7 @@
       <c r="C209" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="D209" s="41"/>
+      <c r="D209" s="32"/>
       <c r="E209" s="12"/>
       <c r="F209" s="12">
         <v>5</v>
@@ -4518,7 +4518,7 @@
       <c r="C210" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="D210" s="41"/>
+      <c r="D210" s="32"/>
       <c r="E210" s="12"/>
       <c r="F210" s="12">
         <v>5</v>
@@ -4530,7 +4530,7 @@
       <c r="C211" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="D211" s="41"/>
+      <c r="D211" s="32"/>
       <c r="E211" s="12"/>
       <c r="F211" s="12">
         <v>5</v>
@@ -4542,7 +4542,7 @@
       <c r="C212" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="D212" s="41"/>
+      <c r="D212" s="32"/>
       <c r="E212" s="12"/>
       <c r="F212" s="12">
         <v>5</v>
@@ -4554,7 +4554,7 @@
       <c r="C213" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="D213" s="41"/>
+      <c r="D213" s="32"/>
       <c r="E213" s="12"/>
       <c r="F213" s="12">
         <v>5</v>
@@ -4564,7 +4564,7 @@
       <c r="A214" s="1"/>
       <c r="B214" s="12"/>
       <c r="C214" s="12"/>
-      <c r="D214" s="42" t="s">
+      <c r="D214" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E214" s="28">
@@ -4591,7 +4591,7 @@
       <c r="C216" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="D216" s="40"/>
+      <c r="D216" s="31"/>
       <c r="E216" s="13"/>
       <c r="F216" s="13">
         <v>5</v>
@@ -4603,7 +4603,7 @@
       <c r="C217" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="D217" s="40"/>
+      <c r="D217" s="31"/>
       <c r="E217" s="13"/>
       <c r="F217" s="13">
         <v>5</v>
@@ -4615,7 +4615,7 @@
       <c r="C218" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D218" s="40"/>
+      <c r="D218" s="31"/>
       <c r="E218" s="13"/>
       <c r="F218" s="13">
         <v>5</v>
@@ -4627,7 +4627,7 @@
       <c r="C219" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="D219" s="40"/>
+      <c r="D219" s="31"/>
       <c r="E219" s="13"/>
       <c r="F219" s="13">
         <v>5</v>
@@ -4639,7 +4639,7 @@
       <c r="C220" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D220" s="40"/>
+      <c r="D220" s="31"/>
       <c r="E220" s="13"/>
       <c r="F220" s="13">
         <v>5</v>
@@ -4651,7 +4651,7 @@
       <c r="C221" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D221" s="40"/>
+      <c r="D221" s="31"/>
       <c r="E221" s="13"/>
       <c r="F221" s="13">
         <v>5</v>
@@ -4663,7 +4663,7 @@
       <c r="C222" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D222" s="40"/>
+      <c r="D222" s="31"/>
       <c r="E222" s="13"/>
       <c r="F222" s="13">
         <v>5</v>
@@ -4675,7 +4675,7 @@
       <c r="C223" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="D223" s="40"/>
+      <c r="D223" s="31"/>
       <c r="E223" s="13"/>
       <c r="F223" s="13">
         <v>5</v>
@@ -4685,7 +4685,7 @@
       <c r="A224" s="1"/>
       <c r="B224" s="13"/>
       <c r="C224" s="13"/>
-      <c r="D224" s="42" t="s">
+      <c r="D224" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E224" s="28">
@@ -4806,7 +4806,7 @@
       <c r="A234" s="1"/>
       <c r="B234" s="14"/>
       <c r="C234" s="14"/>
-      <c r="D234" s="42" t="s">
+      <c r="D234" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E234" s="28">
@@ -4835,7 +4835,7 @@
       <c r="C236" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D236" s="40"/>
+      <c r="D236" s="31"/>
       <c r="E236" s="13"/>
       <c r="F236" s="13">
         <v>10</v>
@@ -4847,7 +4847,7 @@
       <c r="C237" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D237" s="40"/>
+      <c r="D237" s="31"/>
       <c r="E237" s="13"/>
       <c r="F237" s="13">
         <v>10</v>
@@ -4859,7 +4859,7 @@
       <c r="C238" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D238" s="40"/>
+      <c r="D238" s="31"/>
       <c r="E238" s="13"/>
       <c r="F238" s="13">
         <v>10</v>
@@ -4871,7 +4871,7 @@
       <c r="C239" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D239" s="40"/>
+      <c r="D239" s="31"/>
       <c r="E239" s="13"/>
       <c r="F239" s="13">
         <v>10</v>
@@ -4883,7 +4883,7 @@
       <c r="C240" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="D240" s="40"/>
+      <c r="D240" s="31"/>
       <c r="E240" s="13"/>
       <c r="F240" s="13">
         <v>20</v>
@@ -4895,7 +4895,7 @@
       <c r="C241" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D241" s="40"/>
+      <c r="D241" s="31"/>
       <c r="E241" s="13"/>
       <c r="F241" s="13">
         <v>10</v>
@@ -4907,7 +4907,7 @@
       <c r="C242" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D242" s="40"/>
+      <c r="D242" s="31"/>
       <c r="E242" s="13"/>
       <c r="F242" s="13">
         <v>10</v>
@@ -4919,7 +4919,7 @@
       <c r="C243" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D243" s="40"/>
+      <c r="D243" s="31"/>
       <c r="E243" s="13"/>
       <c r="F243" s="13">
         <v>30</v>
@@ -4931,7 +4931,7 @@
       <c r="C244" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="D244" s="40"/>
+      <c r="D244" s="31"/>
       <c r="E244" s="13"/>
       <c r="F244" s="13">
         <v>10</v>
@@ -4941,7 +4941,7 @@
       <c r="A245" s="13"/>
       <c r="B245" s="13"/>
       <c r="C245" s="13"/>
-      <c r="D245" s="42" t="s">
+      <c r="D245" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E245" s="28">
@@ -4953,7 +4953,7 @@
       <c r="A246" s="25"/>
       <c r="B246" s="25"/>
       <c r="C246" s="25"/>
-      <c r="D246" s="45"/>
+      <c r="D246" s="36"/>
       <c r="E246" s="26">
         <f>SUM(E236:E244)*E245</f>
         <v>0</v>
@@ -4967,7 +4967,7 @@
       <c r="A247" s="25"/>
       <c r="B247" s="25"/>
       <c r="C247" s="25"/>
-      <c r="D247" s="45"/>
+      <c r="D247" s="36"/>
       <c r="E247" s="25"/>
       <c r="F247" s="25"/>
     </row>
@@ -4984,7 +4984,7 @@
         <v>205</v>
       </c>
       <c r="C249" s="12"/>
-      <c r="D249" s="41"/>
+      <c r="D249" s="32"/>
       <c r="E249" s="12"/>
       <c r="F249" s="12">
         <v>5</v>
@@ -4998,7 +4998,7 @@
         <v>65</v>
       </c>
       <c r="C250" s="12"/>
-      <c r="D250" s="41"/>
+      <c r="D250" s="32"/>
       <c r="E250" s="12"/>
       <c r="F250" s="12">
         <v>10</v>
@@ -5010,7 +5010,7 @@
         <v>50</v>
       </c>
       <c r="C251" s="12"/>
-      <c r="D251" s="41"/>
+      <c r="D251" s="32"/>
       <c r="E251" s="12"/>
       <c r="F251" s="12">
         <v>10</v>
@@ -5022,7 +5022,7 @@
         <v>207</v>
       </c>
       <c r="C252" s="12"/>
-      <c r="D252" s="41"/>
+      <c r="D252" s="32"/>
       <c r="E252" s="12"/>
       <c r="F252" s="12">
         <v>5</v>
@@ -5034,7 +5034,7 @@
         <v>51</v>
       </c>
       <c r="C253" s="12"/>
-      <c r="D253" s="41"/>
+      <c r="D253" s="32"/>
       <c r="E253" s="12"/>
       <c r="F253" s="12">
         <v>5</v>
@@ -5046,7 +5046,7 @@
         <v>234</v>
       </c>
       <c r="C254" s="12"/>
-      <c r="D254" s="41"/>
+      <c r="D254" s="32"/>
       <c r="E254" s="12"/>
       <c r="F254" s="12">
         <v>5</v>
@@ -5056,7 +5056,7 @@
       <c r="A255" s="11"/>
       <c r="B255" s="12"/>
       <c r="C255" s="12"/>
-      <c r="D255" s="42" t="s">
+      <c r="D255" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E255" s="28">
@@ -5083,12 +5083,12 @@
       <c r="C257" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="D257" s="41"/>
+      <c r="D257" s="32"/>
       <c r="E257" s="12"/>
       <c r="F257" s="12">
         <v>5</v>
       </c>
-      <c r="G257" s="33" t="s">
+      <c r="G257" s="42" t="s">
         <v>109</v>
       </c>
     </row>
@@ -5100,12 +5100,12 @@
       <c r="C258" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="D258" s="41"/>
+      <c r="D258" s="32"/>
       <c r="E258" s="12"/>
       <c r="F258" s="12">
         <v>10</v>
       </c>
-      <c r="G258" s="33"/>
+      <c r="G258" s="42"/>
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A259" s="11" t="s">
@@ -5115,12 +5115,12 @@
       <c r="C259" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D259" s="41"/>
+      <c r="D259" s="32"/>
       <c r="E259" s="12"/>
       <c r="F259" s="12">
         <v>10</v>
       </c>
-      <c r="G259" s="33"/>
+      <c r="G259" s="42"/>
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A260" s="11"/>
@@ -5128,12 +5128,12 @@
       <c r="C260" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="D260" s="41"/>
+      <c r="D260" s="32"/>
       <c r="E260" s="12"/>
       <c r="F260" s="12">
         <v>5</v>
       </c>
-      <c r="G260" s="33"/>
+      <c r="G260" s="42"/>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A261" s="11"/>
@@ -5141,12 +5141,12 @@
       <c r="C261" s="12" t="s">
         <v>329</v>
       </c>
-      <c r="D261" s="41"/>
+      <c r="D261" s="32"/>
       <c r="E261" s="12"/>
       <c r="F261" s="12">
         <v>5</v>
       </c>
-      <c r="G261" s="33"/>
+      <c r="G261" s="42"/>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A262" s="11"/>
@@ -5154,25 +5154,25 @@
       <c r="C262" s="12" t="s">
         <v>328</v>
       </c>
-      <c r="D262" s="41"/>
+      <c r="D262" s="32"/>
       <c r="E262" s="12"/>
       <c r="F262" s="12">
         <v>5</v>
       </c>
-      <c r="G262" s="33"/>
+      <c r="G262" s="42"/>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A263" s="11"/>
       <c r="B263" s="12"/>
       <c r="C263" s="12"/>
-      <c r="D263" s="42" t="s">
+      <c r="D263" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E263" s="28">
         <v>1</v>
       </c>
       <c r="F263" s="12"/>
-      <c r="G263" s="33"/>
+      <c r="G263" s="42"/>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A264" s="1"/>
@@ -5198,7 +5198,7 @@
       <c r="C266" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D266" s="44"/>
+      <c r="D266" s="35"/>
       <c r="E266" s="8"/>
       <c r="F266" s="8"/>
     </row>
@@ -5208,7 +5208,7 @@
       <c r="C267" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D267" s="44"/>
+      <c r="D267" s="35"/>
       <c r="E267" s="8"/>
       <c r="F267" s="8">
         <v>5</v>
@@ -5220,7 +5220,7 @@
       <c r="C268" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D268" s="44"/>
+      <c r="D268" s="35"/>
       <c r="E268" s="8"/>
       <c r="F268" s="8"/>
     </row>
@@ -5230,7 +5230,7 @@
       <c r="C269" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D269" s="44"/>
+      <c r="D269" s="35"/>
       <c r="E269" s="8"/>
       <c r="F269" s="8"/>
     </row>
@@ -5240,7 +5240,7 @@
       <c r="C270" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="D270" s="44"/>
+      <c r="D270" s="35"/>
       <c r="E270" s="8"/>
       <c r="F270" s="8">
         <v>2</v>
@@ -5261,7 +5261,7 @@
       <c r="C273" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="D273" s="41" t="s">
+      <c r="D273" s="32" t="s">
         <v>39</v>
       </c>
       <c r="E273" s="12"/>
@@ -5273,7 +5273,7 @@
       <c r="A274" s="12"/>
       <c r="B274" s="12"/>
       <c r="C274" s="12"/>
-      <c r="D274" s="41" t="s">
+      <c r="D274" s="32" t="s">
         <v>101</v>
       </c>
       <c r="E274" s="12"/>
@@ -5285,7 +5285,7 @@
       <c r="A275" s="12"/>
       <c r="B275" s="12"/>
       <c r="C275" s="12"/>
-      <c r="D275" s="41" t="s">
+      <c r="D275" s="32" t="s">
         <v>286</v>
       </c>
       <c r="E275" s="12"/>
@@ -5297,7 +5297,7 @@
       <c r="A276" s="12"/>
       <c r="B276" s="12"/>
       <c r="C276" s="12"/>
-      <c r="D276" s="41" t="s">
+      <c r="D276" s="32" t="s">
         <v>102</v>
       </c>
       <c r="E276" s="12"/>
@@ -5309,7 +5309,7 @@
       <c r="A277" s="12"/>
       <c r="B277" s="12"/>
       <c r="C277" s="12"/>
-      <c r="D277" s="41" t="s">
+      <c r="D277" s="32" t="s">
         <v>288</v>
       </c>
       <c r="E277" s="12"/>
@@ -5321,7 +5321,7 @@
       <c r="A278" s="12"/>
       <c r="B278" s="12"/>
       <c r="C278" s="12"/>
-      <c r="D278" s="41" t="s">
+      <c r="D278" s="32" t="s">
         <v>287</v>
       </c>
       <c r="E278" s="12"/>
@@ -5335,7 +5335,7 @@
       <c r="C279" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="D279" s="41" t="s">
+      <c r="D279" s="32" t="s">
         <v>290</v>
       </c>
       <c r="E279" s="12"/>
@@ -5347,7 +5347,7 @@
       <c r="A280" s="12"/>
       <c r="B280" s="12"/>
       <c r="C280" s="12"/>
-      <c r="D280" s="41" t="s">
+      <c r="D280" s="32" t="s">
         <v>291</v>
       </c>
       <c r="E280" s="12"/>
@@ -5359,7 +5359,7 @@
       <c r="A281" s="12"/>
       <c r="B281" s="12"/>
       <c r="C281" s="12"/>
-      <c r="D281" s="41" t="s">
+      <c r="D281" s="32" t="s">
         <v>20</v>
       </c>
       <c r="E281" s="12"/>
@@ -5371,7 +5371,7 @@
       <c r="A282" s="12"/>
       <c r="B282" s="12"/>
       <c r="C282" s="12"/>
-      <c r="D282" s="41" t="s">
+      <c r="D282" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E282" s="12"/>
@@ -5383,7 +5383,7 @@
       <c r="A283" s="12"/>
       <c r="B283" s="12"/>
       <c r="C283" s="12"/>
-      <c r="D283" s="41" t="s">
+      <c r="D283" s="32" t="s">
         <v>292</v>
       </c>
       <c r="E283" s="12"/>
@@ -5395,7 +5395,7 @@
       <c r="A284" s="12"/>
       <c r="B284" s="12"/>
       <c r="C284" s="12"/>
-      <c r="D284" s="42" t="s">
+      <c r="D284" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E284" s="28">
@@ -5421,7 +5421,7 @@
         <v>74</v>
       </c>
       <c r="C286" s="8"/>
-      <c r="D286" s="44"/>
+      <c r="D286" s="35"/>
       <c r="E286" s="8"/>
       <c r="F286" s="8">
         <v>5</v>
@@ -5435,7 +5435,7 @@
       <c r="C287" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="D287" s="44"/>
+      <c r="D287" s="35"/>
       <c r="E287" s="8"/>
       <c r="F287" s="8">
         <v>5</v>
@@ -5447,7 +5447,7 @@
       <c r="C288" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D288" s="44"/>
+      <c r="D288" s="35"/>
       <c r="E288" s="8"/>
       <c r="F288" s="8">
         <v>5</v>
@@ -5459,7 +5459,7 @@
       <c r="C289" s="8" t="s">
         <v>295</v>
       </c>
-      <c r="D289" s="44"/>
+      <c r="D289" s="35"/>
       <c r="E289" s="8"/>
       <c r="F289" s="8">
         <v>5</v>
@@ -5471,7 +5471,7 @@
       <c r="C290" s="8" t="s">
         <v>296</v>
       </c>
-      <c r="D290" s="44"/>
+      <c r="D290" s="35"/>
       <c r="E290" s="8"/>
       <c r="F290" s="8">
         <v>5</v>
@@ -5483,7 +5483,7 @@
       <c r="C291" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="D291" s="44"/>
+      <c r="D291" s="35"/>
       <c r="E291" s="8"/>
       <c r="F291" s="8">
         <v>5</v>
@@ -5495,7 +5495,7 @@
       <c r="C292" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="D292" s="44"/>
+      <c r="D292" s="35"/>
       <c r="E292" s="8"/>
       <c r="F292" s="8">
         <v>5</v>
@@ -5505,7 +5505,7 @@
       <c r="A293" s="8"/>
       <c r="B293" s="8"/>
       <c r="C293" s="8"/>
-      <c r="D293" s="42" t="s">
+      <c r="D293" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E293" s="28">
@@ -5531,7 +5531,7 @@
         <v>300</v>
       </c>
       <c r="C296" s="8"/>
-      <c r="D296" s="44"/>
+      <c r="D296" s="35"/>
       <c r="E296" s="8"/>
       <c r="F296" s="8">
         <v>5</v>
@@ -5545,7 +5545,7 @@
         <v>302</v>
       </c>
       <c r="C297" s="8"/>
-      <c r="D297" s="44"/>
+      <c r="D297" s="35"/>
       <c r="E297" s="8"/>
       <c r="F297" s="8">
         <v>5</v>
@@ -5557,7 +5557,7 @@
         <v>303</v>
       </c>
       <c r="C298" s="8"/>
-      <c r="D298" s="44"/>
+      <c r="D298" s="35"/>
       <c r="E298" s="8"/>
       <c r="F298" s="8">
         <v>5</v>
@@ -5569,7 +5569,7 @@
         <v>304</v>
       </c>
       <c r="C299" s="8"/>
-      <c r="D299" s="44"/>
+      <c r="D299" s="35"/>
       <c r="E299" s="8"/>
       <c r="F299" s="8">
         <v>5</v>
@@ -5579,7 +5579,7 @@
       <c r="A300" s="8"/>
       <c r="B300" s="8"/>
       <c r="C300" s="8"/>
-      <c r="D300" s="42" t="s">
+      <c r="D300" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E300" s="28">
@@ -5705,7 +5705,7 @@
       <c r="A311" s="14"/>
       <c r="B311" s="14"/>
       <c r="C311" s="14"/>
-      <c r="D311" s="42" t="s">
+      <c r="D311" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E311" s="28">
@@ -5731,7 +5731,7 @@
         <v>311</v>
       </c>
       <c r="C313" s="12"/>
-      <c r="D313" s="41"/>
+      <c r="D313" s="32"/>
       <c r="E313" s="12"/>
       <c r="F313" s="12">
         <v>5</v>
@@ -5743,7 +5743,7 @@
         <v>251</v>
       </c>
       <c r="C314" s="12"/>
-      <c r="D314" s="41"/>
+      <c r="D314" s="32"/>
       <c r="E314" s="12"/>
       <c r="F314" s="12">
         <v>10</v>
@@ -5755,7 +5755,7 @@
         <v>320</v>
       </c>
       <c r="C315" s="12"/>
-      <c r="D315" s="41"/>
+      <c r="D315" s="32"/>
       <c r="E315" s="12" t="s">
         <v>319</v>
       </c>
@@ -5769,7 +5769,7 @@
         <v>312</v>
       </c>
       <c r="C316" s="12"/>
-      <c r="D316" s="41"/>
+      <c r="D316" s="32"/>
       <c r="E316" s="12" t="s">
         <v>319</v>
       </c>
@@ -5783,7 +5783,7 @@
         <v>230</v>
       </c>
       <c r="C317" s="12"/>
-      <c r="D317" s="41"/>
+      <c r="D317" s="32"/>
       <c r="E317" s="12" t="s">
         <v>319</v>
       </c>
@@ -5797,7 +5797,7 @@
         <v>321</v>
       </c>
       <c r="C318" s="12"/>
-      <c r="D318" s="41"/>
+      <c r="D318" s="32"/>
       <c r="E318" s="12" t="s">
         <v>319</v>
       </c>
@@ -5811,7 +5811,7 @@
         <v>322</v>
       </c>
       <c r="C319" s="12"/>
-      <c r="D319" s="41"/>
+      <c r="D319" s="32"/>
       <c r="E319" s="12"/>
       <c r="F319" s="12">
         <v>5</v>
@@ -5823,7 +5823,7 @@
         <v>313</v>
       </c>
       <c r="C320" s="12"/>
-      <c r="D320" s="41"/>
+      <c r="D320" s="32"/>
       <c r="E320" s="12"/>
       <c r="F320" s="12">
         <v>5</v>
@@ -5835,7 +5835,7 @@
         <v>314</v>
       </c>
       <c r="C321" s="12"/>
-      <c r="D321" s="41"/>
+      <c r="D321" s="32"/>
       <c r="E321" s="12"/>
       <c r="F321" s="12">
         <v>5</v>
@@ -5847,7 +5847,7 @@
         <v>40</v>
       </c>
       <c r="C322" s="12"/>
-      <c r="D322" s="41"/>
+      <c r="D322" s="32"/>
       <c r="E322" s="12"/>
       <c r="F322" s="12">
         <v>10</v>
@@ -5857,7 +5857,7 @@
       <c r="A323" s="12"/>
       <c r="B323" s="12"/>
       <c r="C323" s="12"/>
-      <c r="D323" s="42" t="s">
+      <c r="D323" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E323" s="28">
@@ -5883,7 +5883,7 @@
         <v>190</v>
       </c>
       <c r="C326" s="8"/>
-      <c r="D326" s="44"/>
+      <c r="D326" s="35"/>
       <c r="E326" s="8"/>
       <c r="F326" s="8">
         <v>25</v>
@@ -5895,7 +5895,7 @@
         <v>191</v>
       </c>
       <c r="C327" s="8"/>
-      <c r="D327" s="44"/>
+      <c r="D327" s="35"/>
       <c r="E327" s="8"/>
       <c r="F327" s="8">
         <v>25</v>
@@ -5909,7 +5909,7 @@
       <c r="C328" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="D328" s="44"/>
+      <c r="D328" s="35"/>
       <c r="E328" s="8"/>
       <c r="F328" s="8">
         <v>10</v>
@@ -5921,7 +5921,7 @@
       <c r="C329" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D329" s="44"/>
+      <c r="D329" s="35"/>
       <c r="E329" s="8"/>
       <c r="F329" s="8">
         <v>10</v>
@@ -5933,7 +5933,7 @@
       <c r="C330" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="D330" s="44"/>
+      <c r="D330" s="35"/>
       <c r="E330" s="8"/>
       <c r="F330" s="8">
         <v>10</v>
@@ -5945,7 +5945,7 @@
       <c r="C331" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="D331" s="44"/>
+      <c r="D331" s="35"/>
       <c r="E331" s="8"/>
       <c r="F331" s="8">
         <v>10</v>
@@ -5957,7 +5957,7 @@
       <c r="C332" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D332" s="44"/>
+      <c r="D332" s="35"/>
       <c r="E332" s="8"/>
       <c r="F332" s="8">
         <v>10</v>
@@ -5967,7 +5967,7 @@
       <c r="A333" s="7"/>
       <c r="B333" s="8"/>
       <c r="C333" s="8"/>
-      <c r="D333" s="42" t="s">
+      <c r="D333" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E333" s="28">
@@ -5994,7 +5994,7 @@
         <v>13</v>
       </c>
       <c r="C335" s="8"/>
-      <c r="D335" s="44"/>
+      <c r="D335" s="35"/>
       <c r="E335" s="8"/>
       <c r="F335" s="8">
         <v>10</v>
@@ -6006,7 +6006,7 @@
         <v>46</v>
       </c>
       <c r="C336" s="8"/>
-      <c r="D336" s="44"/>
+      <c r="D336" s="35"/>
       <c r="E336" s="8"/>
       <c r="F336" s="8">
         <v>5</v>
@@ -6018,7 +6018,7 @@
         <v>358</v>
       </c>
       <c r="C337" s="8"/>
-      <c r="D337" s="44"/>
+      <c r="D337" s="35"/>
       <c r="E337" s="8"/>
       <c r="F337" s="8">
         <v>15</v>
@@ -6030,7 +6030,7 @@
         <v>169</v>
       </c>
       <c r="C338" s="8"/>
-      <c r="D338" s="44"/>
+      <c r="D338" s="35"/>
       <c r="E338" s="8"/>
       <c r="F338" s="8">
         <v>5</v>
@@ -6042,7 +6042,7 @@
         <v>77</v>
       </c>
       <c r="C339" s="8"/>
-      <c r="D339" s="44"/>
+      <c r="D339" s="35"/>
       <c r="E339" s="8"/>
       <c r="F339" s="8">
         <v>5</v>
@@ -6054,7 +6054,7 @@
         <v>79</v>
       </c>
       <c r="C340" s="8"/>
-      <c r="D340" s="44"/>
+      <c r="D340" s="35"/>
       <c r="E340" s="8"/>
       <c r="F340" s="8">
         <v>25</v>
@@ -6068,7 +6068,7 @@
       <c r="C341" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="D341" s="44"/>
+      <c r="D341" s="35"/>
       <c r="E341" s="8"/>
       <c r="F341" s="8">
         <v>5</v>
@@ -6080,7 +6080,7 @@
       <c r="C342" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D342" s="44"/>
+      <c r="D342" s="35"/>
       <c r="E342" s="8"/>
       <c r="F342" s="8">
         <v>10</v>
@@ -6092,7 +6092,7 @@
       <c r="C343" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D343" s="44"/>
+      <c r="D343" s="35"/>
       <c r="E343" s="8"/>
       <c r="F343" s="8">
         <v>25</v>
@@ -6104,7 +6104,7 @@
       <c r="C344" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D344" s="44"/>
+      <c r="D344" s="35"/>
       <c r="E344" s="8"/>
       <c r="F344" s="8">
         <v>20</v>
@@ -6116,7 +6116,7 @@
       <c r="C345" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="D345" s="44"/>
+      <c r="D345" s="35"/>
       <c r="E345" s="8"/>
       <c r="F345" s="8">
         <v>20</v>
@@ -6128,7 +6128,7 @@
       <c r="C346" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D346" s="44" t="s">
+      <c r="D346" s="35" t="s">
         <v>69</v>
       </c>
       <c r="E346" s="8"/>
@@ -6140,7 +6140,7 @@
       <c r="A347" s="7"/>
       <c r="B347" s="7"/>
       <c r="C347" s="8"/>
-      <c r="D347" s="44" t="s">
+      <c r="D347" s="35" t="s">
         <v>70</v>
       </c>
       <c r="E347" s="8"/>
@@ -6152,7 +6152,7 @@
       <c r="A348" s="7"/>
       <c r="B348" s="7"/>
       <c r="C348" s="8"/>
-      <c r="D348" s="44" t="s">
+      <c r="D348" s="35" t="s">
         <v>71</v>
       </c>
       <c r="E348" s="8"/>
@@ -6164,7 +6164,7 @@
       <c r="A349" s="7"/>
       <c r="B349" s="7"/>
       <c r="C349" s="8"/>
-      <c r="D349" s="44" t="s">
+      <c r="D349" s="35" t="s">
         <v>54</v>
       </c>
       <c r="E349" s="8"/>
@@ -6176,7 +6176,7 @@
       <c r="A350" s="7"/>
       <c r="B350" s="7"/>
       <c r="C350" s="8"/>
-      <c r="D350" s="44" t="s">
+      <c r="D350" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E350" s="8"/>
@@ -6188,7 +6188,7 @@
       <c r="A351" s="7"/>
       <c r="B351" s="7"/>
       <c r="C351" s="8"/>
-      <c r="D351" s="42" t="s">
+      <c r="D351" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E351" s="28">
@@ -6219,7 +6219,7 @@
         <v>221</v>
       </c>
       <c r="C354" s="13"/>
-      <c r="D354" s="40"/>
+      <c r="D354" s="31"/>
       <c r="E354" s="13"/>
       <c r="F354" s="13">
         <v>10</v>
@@ -6233,7 +6233,7 @@
       <c r="C355" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="D355" s="40"/>
+      <c r="D355" s="31"/>
       <c r="E355" s="13"/>
       <c r="F355" s="13">
         <v>30</v>
@@ -6245,7 +6245,7 @@
       <c r="C356" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="D356" s="40"/>
+      <c r="D356" s="31"/>
       <c r="E356" s="13"/>
       <c r="F356" s="13">
         <v>30</v>
@@ -6257,7 +6257,7 @@
       <c r="C357" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="D357" s="40"/>
+      <c r="D357" s="31"/>
       <c r="E357" s="13"/>
       <c r="F357" s="13">
         <v>30</v>
@@ -6271,7 +6271,7 @@
       <c r="C358" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="D358" s="40"/>
+      <c r="D358" s="31"/>
       <c r="E358" s="13"/>
       <c r="F358" s="13">
         <v>30</v>
@@ -6283,7 +6283,7 @@
       <c r="C359" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="D359" s="40"/>
+      <c r="D359" s="31"/>
       <c r="E359" s="13"/>
       <c r="F359" s="13">
         <v>30</v>
@@ -6295,7 +6295,7 @@
       <c r="C360" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="D360" s="40"/>
+      <c r="D360" s="31"/>
       <c r="E360" s="13"/>
       <c r="F360" s="13">
         <v>30</v>
@@ -6305,7 +6305,7 @@
       <c r="A361" s="13"/>
       <c r="B361" s="13"/>
       <c r="C361" s="13"/>
-      <c r="D361" s="42" t="s">
+      <c r="D361" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E361" s="28">
@@ -6327,7 +6327,7 @@
       <c r="A363" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="D363" s="46"/>
+      <c r="D363" s="37"/>
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A364" s="15" t="s">
@@ -6337,7 +6337,7 @@
       <c r="C364" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="D364" s="40"/>
+      <c r="D364" s="31"/>
       <c r="E364" s="13">
         <v>0</v>
       </c>
@@ -6351,7 +6351,7 @@
       <c r="C365" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="D365" s="40"/>
+      <c r="D365" s="31"/>
       <c r="E365" s="13">
         <v>0</v>
       </c>
@@ -6365,7 +6365,7 @@
       <c r="C366" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="D366" s="40"/>
+      <c r="D366" s="31"/>
       <c r="E366" s="13">
         <v>0</v>
       </c>
@@ -6379,7 +6379,7 @@
       <c r="C367" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="D367" s="40"/>
+      <c r="D367" s="31"/>
       <c r="E367" s="13">
         <v>0</v>
       </c>
@@ -6393,7 +6393,7 @@
       <c r="C368" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="D368" s="40"/>
+      <c r="D368" s="31"/>
       <c r="E368" s="13">
         <v>0</v>
       </c>
@@ -6407,7 +6407,7 @@
       <c r="C369" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="D369" s="40"/>
+      <c r="D369" s="31"/>
       <c r="E369" s="13">
         <v>0</v>
       </c>
@@ -6419,7 +6419,7 @@
       <c r="A370" s="13"/>
       <c r="B370" s="13"/>
       <c r="C370" s="13"/>
-      <c r="D370" s="42" t="s">
+      <c r="D370" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E370" s="28">
@@ -6445,7 +6445,7 @@
         <v>356</v>
       </c>
       <c r="C372" s="17"/>
-      <c r="D372" s="40"/>
+      <c r="D372" s="31"/>
       <c r="E372" s="13"/>
       <c r="F372" s="13">
         <v>10</v>
@@ -6457,7 +6457,7 @@
         <v>77</v>
       </c>
       <c r="C373" s="17"/>
-      <c r="D373" s="40"/>
+      <c r="D373" s="31"/>
       <c r="E373" s="13"/>
       <c r="F373" s="13">
         <v>5</v>
@@ -6469,7 +6469,7 @@
         <v>124</v>
       </c>
       <c r="C374" s="17"/>
-      <c r="D374" s="40"/>
+      <c r="D374" s="31"/>
       <c r="E374" s="13"/>
       <c r="F374" s="13">
         <v>5</v>
@@ -6479,7 +6479,7 @@
       <c r="A375" s="15"/>
       <c r="B375" s="13"/>
       <c r="C375" s="13"/>
-      <c r="D375" s="40"/>
+      <c r="D375" s="31"/>
       <c r="E375" s="13"/>
       <c r="F375" s="13"/>
     </row>
@@ -6491,7 +6491,7 @@
         <v>77</v>
       </c>
       <c r="C376" s="13"/>
-      <c r="D376" s="40"/>
+      <c r="D376" s="31"/>
       <c r="E376" s="13"/>
       <c r="F376" s="13">
         <v>5</v>
@@ -6503,7 +6503,7 @@
         <v>123</v>
       </c>
       <c r="C377" s="13"/>
-      <c r="D377" s="40"/>
+      <c r="D377" s="31"/>
       <c r="E377" s="13"/>
       <c r="F377" s="13">
         <v>5</v>
@@ -6515,7 +6515,7 @@
         <v>124</v>
       </c>
       <c r="C378" s="13"/>
-      <c r="D378" s="40"/>
+      <c r="D378" s="31"/>
       <c r="E378" s="13"/>
       <c r="F378" s="13">
         <v>5</v>
@@ -6525,7 +6525,7 @@
       <c r="A379" s="15"/>
       <c r="B379" s="13"/>
       <c r="C379" s="13"/>
-      <c r="D379" s="40"/>
+      <c r="D379" s="31"/>
       <c r="E379" s="13"/>
       <c r="F379" s="13"/>
     </row>
@@ -6537,7 +6537,7 @@
         <v>77</v>
       </c>
       <c r="C380" s="13"/>
-      <c r="D380" s="40"/>
+      <c r="D380" s="31"/>
       <c r="E380" s="13"/>
       <c r="F380" s="13">
         <v>5</v>
@@ -6549,7 +6549,7 @@
         <v>123</v>
       </c>
       <c r="C381" s="13"/>
-      <c r="D381" s="40"/>
+      <c r="D381" s="31"/>
       <c r="E381" s="13"/>
       <c r="F381" s="13">
         <v>5</v>
@@ -6561,7 +6561,7 @@
         <v>124</v>
       </c>
       <c r="C382" s="13"/>
-      <c r="D382" s="40"/>
+      <c r="D382" s="31"/>
       <c r="E382" s="13"/>
       <c r="F382" s="13">
         <v>5</v>
@@ -6571,7 +6571,7 @@
       <c r="A383" s="15"/>
       <c r="B383" s="13"/>
       <c r="C383" s="13"/>
-      <c r="D383" s="42" t="s">
+      <c r="D383" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E383" s="28">
@@ -6624,7 +6624,7 @@
       <c r="A387" s="16"/>
       <c r="B387" s="14"/>
       <c r="C387" s="14"/>
-      <c r="D387" s="42" t="s">
+      <c r="D387" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E387" s="28">
@@ -6658,7 +6658,7 @@
         <v>105</v>
       </c>
       <c r="C392" s="12"/>
-      <c r="D392" s="41"/>
+      <c r="D392" s="32"/>
       <c r="E392" s="12"/>
       <c r="F392" s="12">
         <v>10</v>
@@ -6670,7 +6670,7 @@
         <v>106</v>
       </c>
       <c r="C393" s="12"/>
-      <c r="D393" s="41"/>
+      <c r="D393" s="32"/>
       <c r="E393" s="12"/>
       <c r="F393" s="12">
         <v>10</v>
@@ -6682,7 +6682,7 @@
         <v>107</v>
       </c>
       <c r="C394" s="12"/>
-      <c r="D394" s="41"/>
+      <c r="D394" s="32"/>
       <c r="E394" s="12"/>
       <c r="F394" s="12">
         <v>10</v>
@@ -6694,7 +6694,7 @@
         <v>108</v>
       </c>
       <c r="C395" s="12"/>
-      <c r="D395" s="41"/>
+      <c r="D395" s="32"/>
       <c r="E395" s="12"/>
       <c r="F395" s="12">
         <v>10</v>
@@ -6706,7 +6706,7 @@
       </c>
       <c r="B396" s="12"/>
       <c r="C396" s="12"/>
-      <c r="D396" s="41"/>
+      <c r="D396" s="32"/>
       <c r="E396" s="12"/>
       <c r="F396" s="12"/>
     </row>
@@ -6716,7 +6716,7 @@
         <v>142</v>
       </c>
       <c r="C397" s="12"/>
-      <c r="D397" s="41"/>
+      <c r="D397" s="32"/>
       <c r="E397" s="12"/>
       <c r="F397" s="12">
         <v>5</v>
@@ -6728,7 +6728,7 @@
         <v>143</v>
       </c>
       <c r="C398" s="12"/>
-      <c r="D398" s="41"/>
+      <c r="D398" s="32"/>
       <c r="E398" s="12"/>
       <c r="F398" s="12">
         <v>15</v>
@@ -6740,7 +6740,7 @@
         <v>144</v>
       </c>
       <c r="C399" s="12"/>
-      <c r="D399" s="41"/>
+      <c r="D399" s="32"/>
       <c r="E399" s="12"/>
       <c r="F399" s="12">
         <v>20</v>
@@ -6752,7 +6752,7 @@
         <v>145</v>
       </c>
       <c r="C400" s="12"/>
-      <c r="D400" s="41"/>
+      <c r="D400" s="32"/>
       <c r="E400" s="12"/>
       <c r="F400" s="12">
         <v>5</v>
@@ -6762,7 +6762,7 @@
       <c r="A401" s="12"/>
       <c r="B401" s="12"/>
       <c r="C401" s="12"/>
-      <c r="D401" s="41"/>
+      <c r="D401" s="32"/>
       <c r="E401" s="12"/>
       <c r="F401" s="12"/>
     </row>
@@ -6774,7 +6774,7 @@
         <v>147</v>
       </c>
       <c r="C402" s="12"/>
-      <c r="D402" s="41"/>
+      <c r="D402" s="32"/>
       <c r="E402" s="12"/>
       <c r="F402" s="12">
         <v>5</v>
@@ -6786,7 +6786,7 @@
         <v>148</v>
       </c>
       <c r="C403" s="12"/>
-      <c r="D403" s="41"/>
+      <c r="D403" s="32"/>
       <c r="E403" s="12"/>
       <c r="F403" s="12">
         <v>15</v>
@@ -6798,7 +6798,7 @@
         <v>149</v>
       </c>
       <c r="C404" s="12"/>
-      <c r="D404" s="41"/>
+      <c r="D404" s="32"/>
       <c r="E404" s="12"/>
       <c r="F404" s="12">
         <v>15</v>
@@ -6808,7 +6808,7 @@
       <c r="A405" s="12"/>
       <c r="B405" s="12"/>
       <c r="C405" s="12"/>
-      <c r="D405" s="42" t="s">
+      <c r="D405" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E405" s="28">
@@ -6841,7 +6841,7 @@
       <c r="C408" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="D408" s="44"/>
+      <c r="D408" s="35"/>
       <c r="E408" s="8"/>
       <c r="F408" s="8">
         <v>2</v>
@@ -6853,7 +6853,7 @@
       <c r="C409" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="D409" s="44"/>
+      <c r="D409" s="35"/>
       <c r="E409" s="8"/>
       <c r="F409" s="8">
         <v>2</v>
@@ -6865,7 +6865,7 @@
       <c r="C410" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="D410" s="44"/>
+      <c r="D410" s="35"/>
       <c r="E410" s="8"/>
       <c r="F410" s="8">
         <v>2</v>
@@ -6877,7 +6877,7 @@
       <c r="C411" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="D411" s="44"/>
+      <c r="D411" s="35"/>
       <c r="E411" s="8"/>
       <c r="F411" s="8">
         <v>2</v>
@@ -6889,7 +6889,7 @@
       <c r="C412" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="D412" s="44"/>
+      <c r="D412" s="35"/>
       <c r="E412" s="8"/>
       <c r="F412" s="8">
         <v>2</v>
@@ -6901,7 +6901,7 @@
         <v>13</v>
       </c>
       <c r="C413" s="8"/>
-      <c r="D413" s="44"/>
+      <c r="D413" s="35"/>
       <c r="E413" s="8"/>
       <c r="F413" s="8">
         <v>5</v>
@@ -6913,7 +6913,7 @@
         <v>43</v>
       </c>
       <c r="C414" s="8"/>
-      <c r="D414" s="44"/>
+      <c r="D414" s="35"/>
       <c r="E414" s="8"/>
       <c r="F414" s="8">
         <v>5</v>
@@ -6925,7 +6925,7 @@
         <v>80</v>
       </c>
       <c r="C415" s="8"/>
-      <c r="D415" s="44"/>
+      <c r="D415" s="35"/>
       <c r="E415" s="8"/>
       <c r="F415" s="8">
         <v>5</v>
@@ -6937,7 +6937,7 @@
         <v>99</v>
       </c>
       <c r="C416" s="8"/>
-      <c r="D416" s="44"/>
+      <c r="D416" s="35"/>
       <c r="E416" s="8"/>
       <c r="F416" s="8">
         <v>5</v>
@@ -6947,7 +6947,7 @@
       <c r="A417" s="8"/>
       <c r="B417" s="8"/>
       <c r="C417" s="8"/>
-      <c r="D417" s="42" t="s">
+      <c r="D417" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E417" s="28">
@@ -7079,7 +7079,7 @@
       <c r="A428" s="14"/>
       <c r="B428" s="14"/>
       <c r="C428" s="14"/>
-      <c r="D428" s="42" t="s">
+      <c r="D428" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E428" s="28">
@@ -7105,7 +7105,7 @@
         <v>159</v>
       </c>
       <c r="C430" s="8"/>
-      <c r="D430" s="44"/>
+      <c r="D430" s="35"/>
       <c r="E430" s="8"/>
       <c r="F430" s="8">
         <v>3</v>
@@ -7117,7 +7117,7 @@
         <v>160</v>
       </c>
       <c r="C431" s="8"/>
-      <c r="D431" s="44"/>
+      <c r="D431" s="35"/>
       <c r="E431" s="8"/>
       <c r="F431" s="8">
         <v>5</v>
@@ -7129,7 +7129,7 @@
         <v>8</v>
       </c>
       <c r="C432" s="8"/>
-      <c r="D432" s="44"/>
+      <c r="D432" s="35"/>
       <c r="E432" s="8"/>
       <c r="F432" s="8">
         <v>3</v>
@@ -7141,7 +7141,7 @@
         <v>161</v>
       </c>
       <c r="C433" s="8"/>
-      <c r="D433" s="44"/>
+      <c r="D433" s="35"/>
       <c r="E433" s="8"/>
       <c r="F433" s="8">
         <v>3</v>
@@ -7153,7 +7153,7 @@
         <v>162</v>
       </c>
       <c r="C434" s="8"/>
-      <c r="D434" s="44"/>
+      <c r="D434" s="35"/>
       <c r="E434" s="8"/>
       <c r="F434" s="8">
         <v>3</v>
@@ -7165,7 +7165,7 @@
         <v>163</v>
       </c>
       <c r="C435" s="8"/>
-      <c r="D435" s="44"/>
+      <c r="D435" s="35"/>
       <c r="E435" s="8"/>
       <c r="F435" s="8">
         <v>3</v>
@@ -7177,7 +7177,7 @@
         <v>164</v>
       </c>
       <c r="C436" s="8"/>
-      <c r="D436" s="44"/>
+      <c r="D436" s="35"/>
       <c r="E436" s="8"/>
       <c r="F436" s="8">
         <v>3</v>
@@ -7187,7 +7187,7 @@
       <c r="A437" s="8"/>
       <c r="B437" s="8"/>
       <c r="C437" s="8"/>
-      <c r="D437" s="42" t="s">
+      <c r="D437" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E437" s="28">
@@ -7213,7 +7213,7 @@
       <c r="C439" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="D439" s="44" t="s">
+      <c r="D439" s="35" t="s">
         <v>173</v>
       </c>
       <c r="E439" s="8"/>
@@ -7221,11 +7221,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="440" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A440" s="7"/>
       <c r="B440" s="7"/>
       <c r="C440" s="8"/>
-      <c r="D440" s="44" t="s">
+      <c r="D440" s="35" t="s">
         <v>174</v>
       </c>
       <c r="E440" s="8"/>
@@ -7233,11 +7233,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="441" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A441" s="7"/>
       <c r="B441" s="7"/>
       <c r="C441" s="8"/>
-      <c r="D441" s="44" t="s">
+      <c r="D441" s="35" t="s">
         <v>175</v>
       </c>
       <c r="E441" s="8"/>
@@ -7251,7 +7251,7 @@
       <c r="C442" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="D442" s="44" t="s">
+      <c r="D442" s="35" t="s">
         <v>177</v>
       </c>
       <c r="E442" s="8"/>
@@ -7263,7 +7263,7 @@
       <c r="A443" s="7"/>
       <c r="B443" s="7"/>
       <c r="C443" s="8"/>
-      <c r="D443" s="44" t="s">
+      <c r="D443" s="35" t="s">
         <v>178</v>
       </c>
       <c r="E443" s="8"/>
@@ -7275,7 +7275,7 @@
       <c r="A444" s="7"/>
       <c r="B444" s="7"/>
       <c r="C444" s="8"/>
-      <c r="D444" s="44" t="s">
+      <c r="D444" s="35" t="s">
         <v>179</v>
       </c>
       <c r="E444" s="8"/>
@@ -7287,7 +7287,7 @@
       <c r="A445" s="7"/>
       <c r="B445" s="7"/>
       <c r="C445" s="8"/>
-      <c r="D445" s="44" t="s">
+      <c r="D445" s="35" t="s">
         <v>180</v>
       </c>
       <c r="E445" s="8"/>
@@ -7299,7 +7299,7 @@
       <c r="A446" s="7"/>
       <c r="B446" s="7"/>
       <c r="C446" s="8"/>
-      <c r="D446" s="44" t="s">
+      <c r="D446" s="35" t="s">
         <v>181</v>
       </c>
       <c r="E446" s="8"/>
@@ -7332,7 +7332,7 @@
       <c r="C449" s="8" t="s">
         <v>316</v>
       </c>
-      <c r="D449" s="44"/>
+      <c r="D449" s="35"/>
       <c r="E449" s="8"/>
       <c r="F449" s="8">
         <v>10</v>
@@ -7344,7 +7344,7 @@
       <c r="C450" s="8" t="s">
         <v>364</v>
       </c>
-      <c r="D450" s="44"/>
+      <c r="D450" s="35"/>
       <c r="E450" s="8"/>
       <c r="F450" s="8">
         <v>10</v>
@@ -7358,7 +7358,7 @@
       <c r="C451" s="8" t="s">
         <v>319</v>
       </c>
-      <c r="D451" s="44"/>
+      <c r="D451" s="35"/>
       <c r="E451" s="8"/>
       <c r="F451" s="8"/>
     </row>
@@ -7368,7 +7368,7 @@
       <c r="C452" s="8" t="s">
         <v>365</v>
       </c>
-      <c r="D452" s="44"/>
+      <c r="D452" s="35"/>
       <c r="E452" s="8"/>
       <c r="F452" s="8">
         <v>10</v>
@@ -7380,7 +7380,7 @@
       <c r="C453" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="D453" s="44"/>
+      <c r="D453" s="35"/>
       <c r="E453" s="8"/>
       <c r="F453" s="8">
         <v>10</v>
@@ -7392,7 +7392,7 @@
       <c r="C454" s="8" t="s">
         <v>366</v>
       </c>
-      <c r="D454" s="44"/>
+      <c r="D454" s="35"/>
       <c r="E454" s="8"/>
       <c r="F454" s="8">
         <v>10</v>
@@ -7404,7 +7404,7 @@
       <c r="C455" s="8" t="s">
         <v>367</v>
       </c>
-      <c r="D455" s="44"/>
+      <c r="D455" s="35"/>
       <c r="E455" s="8"/>
       <c r="F455" s="8">
         <v>10</v>
@@ -7414,7 +7414,7 @@
       <c r="A456" s="8"/>
       <c r="B456" s="8"/>
       <c r="C456" s="8"/>
-      <c r="D456" s="42" t="s">
+      <c r="D456" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E456" s="28">
@@ -7444,7 +7444,7 @@
         <v>370</v>
       </c>
       <c r="C459" s="12"/>
-      <c r="D459" s="41"/>
+      <c r="D459" s="32"/>
       <c r="E459" s="12"/>
       <c r="F459" s="12">
         <v>10</v>
@@ -7460,7 +7460,7 @@
       <c r="C460" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="D460" s="41"/>
+      <c r="D460" s="32"/>
       <c r="E460" s="12"/>
       <c r="F460" s="12">
         <v>20</v>
@@ -7472,7 +7472,7 @@
       <c r="C461" s="12" t="s">
         <v>373</v>
       </c>
-      <c r="D461" s="41"/>
+      <c r="D461" s="32"/>
       <c r="E461" s="12"/>
       <c r="F461" s="12">
         <v>20</v>
@@ -7482,7 +7482,7 @@
       <c r="A462" s="11"/>
       <c r="B462" s="12"/>
       <c r="C462" s="12"/>
-      <c r="D462" s="42" t="s">
+      <c r="D462" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E462" s="28">
@@ -7519,7 +7519,7 @@
       <c r="C466" s="13" t="s">
         <v>351</v>
       </c>
-      <c r="D466" s="40"/>
+      <c r="D466" s="31"/>
       <c r="E466" s="13"/>
       <c r="F466" s="13">
         <v>10</v>
@@ -7533,7 +7533,7 @@
         <v>7</v>
       </c>
       <c r="C467" s="13"/>
-      <c r="D467" s="40"/>
+      <c r="D467" s="31"/>
       <c r="E467" s="13"/>
       <c r="F467" s="13">
         <v>10</v>
@@ -7547,7 +7547,7 @@
         <v>349</v>
       </c>
       <c r="C468" s="13"/>
-      <c r="D468" s="40"/>
+      <c r="D468" s="31"/>
       <c r="E468" s="13"/>
       <c r="F468" s="13">
         <v>20</v>
@@ -7559,7 +7559,7 @@
         <v>350</v>
       </c>
       <c r="C469" s="13"/>
-      <c r="D469" s="40"/>
+      <c r="D469" s="31"/>
       <c r="E469" s="13"/>
       <c r="F469" s="13">
         <v>10</v>
@@ -7569,7 +7569,7 @@
       <c r="A470" s="13"/>
       <c r="B470" s="13"/>
       <c r="C470" s="13"/>
-      <c r="D470" s="42" t="s">
+      <c r="D470" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E470" s="28">
@@ -7633,7 +7633,7 @@
       <c r="A476" s="14"/>
       <c r="B476" s="14"/>
       <c r="C476" s="14"/>
-      <c r="D476" s="42" t="s">
+      <c r="D476" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E476" s="28">
@@ -7661,7 +7661,7 @@
       <c r="C478" s="12" t="s">
         <v>351</v>
       </c>
-      <c r="D478" s="41"/>
+      <c r="D478" s="32"/>
       <c r="E478" s="12"/>
       <c r="F478" s="12">
         <v>10</v>
@@ -7675,7 +7675,7 @@
         <v>352</v>
       </c>
       <c r="C479" s="12"/>
-      <c r="D479" s="41"/>
+      <c r="D479" s="32"/>
       <c r="E479" s="12"/>
       <c r="F479" s="12">
         <v>20</v>
@@ -7687,7 +7687,7 @@
         <v>354</v>
       </c>
       <c r="C480" s="12"/>
-      <c r="D480" s="41"/>
+      <c r="D480" s="32"/>
       <c r="E480" s="12"/>
       <c r="F480" s="12">
         <v>40</v>
@@ -7697,7 +7697,7 @@
       <c r="A481" s="12"/>
       <c r="B481" s="12"/>
       <c r="C481" s="12"/>
-      <c r="D481" s="42" t="s">
+      <c r="D481" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E481" s="28">
@@ -7860,7 +7860,7 @@
       <c r="A499" s="14"/>
       <c r="B499" s="14"/>
       <c r="C499" s="14"/>
-      <c r="D499" s="42" t="s">
+      <c r="D499" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E499" s="28">
@@ -7886,7 +7886,7 @@
         <v>266</v>
       </c>
       <c r="C502" s="12"/>
-      <c r="D502" s="41"/>
+      <c r="D502" s="32"/>
       <c r="E502" s="12"/>
       <c r="F502" s="12">
         <v>10</v>
@@ -7900,7 +7900,7 @@
         <v>120</v>
       </c>
       <c r="C503" s="12"/>
-      <c r="D503" s="41"/>
+      <c r="D503" s="32"/>
       <c r="E503" s="12"/>
       <c r="F503" s="12">
         <v>5</v>
@@ -7912,7 +7912,7 @@
         <v>268</v>
       </c>
       <c r="C504" s="12"/>
-      <c r="D504" s="41"/>
+      <c r="D504" s="32"/>
       <c r="E504" s="12"/>
       <c r="F504" s="12">
         <v>5</v>
@@ -7924,7 +7924,7 @@
         <v>267</v>
       </c>
       <c r="C505" s="12"/>
-      <c r="D505" s="41"/>
+      <c r="D505" s="32"/>
       <c r="E505" s="12"/>
       <c r="F505" s="12">
         <v>5</v>
@@ -7936,7 +7936,7 @@
         <v>269</v>
       </c>
       <c r="C506" s="12"/>
-      <c r="D506" s="41"/>
+      <c r="D506" s="32"/>
       <c r="E506" s="12"/>
       <c r="F506" s="12">
         <v>5</v>
@@ -7948,7 +7948,7 @@
         <v>271</v>
       </c>
       <c r="C507" s="12"/>
-      <c r="D507" s="41"/>
+      <c r="D507" s="32"/>
       <c r="E507" s="12"/>
       <c r="F507" s="12">
         <v>5</v>
@@ -7960,7 +7960,7 @@
         <v>272</v>
       </c>
       <c r="C508" s="12"/>
-      <c r="D508" s="41"/>
+      <c r="D508" s="32"/>
       <c r="E508" s="12"/>
       <c r="F508" s="12">
         <v>5</v>
@@ -7972,7 +7972,7 @@
         <v>26</v>
       </c>
       <c r="C509" s="12"/>
-      <c r="D509" s="41"/>
+      <c r="D509" s="32"/>
       <c r="E509" s="12"/>
       <c r="F509" s="12">
         <v>5</v>
@@ -7984,7 +7984,7 @@
         <v>27</v>
       </c>
       <c r="C510" s="12"/>
-      <c r="D510" s="41"/>
+      <c r="D510" s="32"/>
       <c r="E510" s="12"/>
       <c r="F510" s="12">
         <v>5</v>
@@ -7996,7 +7996,7 @@
         <v>273</v>
       </c>
       <c r="C511" s="12"/>
-      <c r="D511" s="41"/>
+      <c r="D511" s="32"/>
       <c r="E511" s="12"/>
       <c r="F511" s="12">
         <v>5</v>
@@ -8008,7 +8008,7 @@
         <v>274</v>
       </c>
       <c r="C512" s="12"/>
-      <c r="D512" s="41"/>
+      <c r="D512" s="32"/>
       <c r="E512" s="12"/>
       <c r="F512" s="12">
         <v>5</v>
@@ -8018,7 +8018,7 @@
       <c r="A513" s="12"/>
       <c r="B513" s="12"/>
       <c r="C513" s="12"/>
-      <c r="D513" s="42" t="s">
+      <c r="D513" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E513" s="28">
@@ -8044,7 +8044,7 @@
         <v>266</v>
       </c>
       <c r="C516" s="13"/>
-      <c r="D516" s="40"/>
+      <c r="D516" s="31"/>
       <c r="E516" s="13"/>
       <c r="F516" s="13">
         <v>10</v>
@@ -8058,7 +8058,7 @@
         <v>120</v>
       </c>
       <c r="C517" s="13"/>
-      <c r="D517" s="40"/>
+      <c r="D517" s="31"/>
       <c r="E517" s="13"/>
       <c r="F517" s="13">
         <v>5</v>
@@ -8070,7 +8070,7 @@
         <v>268</v>
       </c>
       <c r="C518" s="13"/>
-      <c r="D518" s="40"/>
+      <c r="D518" s="31"/>
       <c r="E518" s="13"/>
       <c r="F518" s="13">
         <v>5</v>
@@ -8082,7 +8082,7 @@
         <v>267</v>
       </c>
       <c r="C519" s="13"/>
-      <c r="D519" s="40"/>
+      <c r="D519" s="31"/>
       <c r="E519" s="13"/>
       <c r="F519" s="13">
         <v>5</v>
@@ -8094,7 +8094,7 @@
         <v>269</v>
       </c>
       <c r="C520" s="13"/>
-      <c r="D520" s="40"/>
+      <c r="D520" s="31"/>
       <c r="E520" s="13"/>
       <c r="F520" s="13">
         <v>5</v>
@@ -8106,7 +8106,7 @@
         <v>271</v>
       </c>
       <c r="C521" s="13"/>
-      <c r="D521" s="40"/>
+      <c r="D521" s="31"/>
       <c r="E521" s="13"/>
       <c r="F521" s="13">
         <v>5</v>
@@ -8118,7 +8118,7 @@
         <v>272</v>
       </c>
       <c r="C522" s="13"/>
-      <c r="D522" s="40"/>
+      <c r="D522" s="31"/>
       <c r="E522" s="13"/>
       <c r="F522" s="13">
         <v>5</v>
@@ -8130,7 +8130,7 @@
         <v>26</v>
       </c>
       <c r="C523" s="13"/>
-      <c r="D523" s="40"/>
+      <c r="D523" s="31"/>
       <c r="E523" s="13"/>
       <c r="F523" s="13">
         <v>5</v>
@@ -8142,7 +8142,7 @@
         <v>27</v>
       </c>
       <c r="C524" s="13"/>
-      <c r="D524" s="40"/>
+      <c r="D524" s="31"/>
       <c r="E524" s="13"/>
       <c r="F524" s="13">
         <v>5</v>
@@ -8154,7 +8154,7 @@
         <v>273</v>
       </c>
       <c r="C525" s="13"/>
-      <c r="D525" s="40"/>
+      <c r="D525" s="31"/>
       <c r="E525" s="13"/>
       <c r="F525" s="13">
         <v>5</v>
@@ -8166,7 +8166,7 @@
         <v>274</v>
       </c>
       <c r="C526" s="13"/>
-      <c r="D526" s="40"/>
+      <c r="D526" s="31"/>
       <c r="E526" s="13"/>
       <c r="F526" s="13">
         <v>5</v>
@@ -8176,7 +8176,7 @@
       <c r="A527" s="13"/>
       <c r="B527" s="13"/>
       <c r="C527" s="13"/>
-      <c r="D527" s="42" t="s">
+      <c r="D527" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E527" s="28">
@@ -8275,7 +8275,7 @@
       <c r="A536" s="14"/>
       <c r="B536" s="14"/>
       <c r="C536" s="14"/>
-      <c r="D536" s="42" t="s">
+      <c r="D536" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E536" s="28">
@@ -8299,7 +8299,7 @@
       </c>
       <c r="B539" s="12"/>
       <c r="C539" s="12"/>
-      <c r="D539" s="41"/>
+      <c r="D539" s="32"/>
       <c r="E539" s="12"/>
       <c r="F539" s="12">
         <v>30</v>
@@ -8309,7 +8309,7 @@
       <c r="A540" s="12"/>
       <c r="B540" s="12"/>
       <c r="C540" s="12"/>
-      <c r="D540" s="41"/>
+      <c r="D540" s="32"/>
       <c r="E540" s="12"/>
       <c r="F540" s="12">
         <v>30</v>
@@ -8319,7 +8319,7 @@
       <c r="A541" s="12"/>
       <c r="B541" s="12"/>
       <c r="C541" s="12"/>
-      <c r="D541" s="41"/>
+      <c r="D541" s="32"/>
       <c r="E541" s="12"/>
       <c r="F541" s="12">
         <v>30</v>
@@ -8329,7 +8329,7 @@
       <c r="A542" s="12"/>
       <c r="B542" s="12"/>
       <c r="C542" s="12"/>
-      <c r="D542" s="41"/>
+      <c r="D542" s="32"/>
       <c r="E542" s="12"/>
       <c r="F542" s="12">
         <v>30</v>
@@ -8339,7 +8339,7 @@
       <c r="A543" s="12"/>
       <c r="B543" s="12"/>
       <c r="C543" s="12"/>
-      <c r="D543" s="41"/>
+      <c r="D543" s="32"/>
       <c r="E543" s="12"/>
       <c r="F543" s="12">
         <v>30</v>
@@ -8349,7 +8349,7 @@
       <c r="A544" s="12"/>
       <c r="B544" s="12"/>
       <c r="C544" s="12"/>
-      <c r="D544" s="42" t="s">
+      <c r="D544" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E544" s="28">
@@ -8375,7 +8375,7 @@
         <v>414</v>
       </c>
       <c r="C547" s="13"/>
-      <c r="D547" s="40" t="s">
+      <c r="D547" s="31" t="s">
         <v>415</v>
       </c>
       <c r="E547" s="13"/>
@@ -8389,7 +8389,7 @@
         <v>416</v>
       </c>
       <c r="C548" s="13"/>
-      <c r="D548" s="40" t="s">
+      <c r="D548" s="31" t="s">
         <v>417</v>
       </c>
       <c r="E548" s="13"/>
@@ -8403,7 +8403,7 @@
         <v>419</v>
       </c>
       <c r="C549" s="13"/>
-      <c r="D549" s="40" t="s">
+      <c r="D549" s="31" t="s">
         <v>418</v>
       </c>
       <c r="E549" s="13"/>
@@ -8417,7 +8417,7 @@
         <v>420</v>
       </c>
       <c r="C550" s="13"/>
-      <c r="D550" s="40" t="s">
+      <c r="D550" s="31" t="s">
         <v>421</v>
       </c>
       <c r="E550" s="13"/>
@@ -8431,7 +8431,7 @@
         <v>422</v>
       </c>
       <c r="C551" s="13"/>
-      <c r="D551" s="40" t="s">
+      <c r="D551" s="31" t="s">
         <v>423</v>
       </c>
       <c r="E551" s="13"/>
@@ -8443,7 +8443,7 @@
       <c r="A552" s="13"/>
       <c r="B552" s="13"/>
       <c r="C552" s="13"/>
-      <c r="D552" s="42" t="s">
+      <c r="D552" s="33" t="s">
         <v>389</v>
       </c>
       <c r="E552" s="28">
@@ -8548,7 +8548,7 @@
       </c>
     </row>
     <row r="564" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D564" s="38" t="s">
+      <c r="D564" s="29" t="s">
         <v>262</v>
       </c>
       <c r="G564" t="s">
@@ -8683,11 +8683,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33.6" x14ac:dyDescent="0.65">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="38" t="s">
         <v>392</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -8695,11 +8695,11 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="39" t="s">
         <v>393</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -9515,7 +9515,7 @@
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A96" s="36" t="s">
+      <c r="A96" s="45" t="s">
         <v>62</v>
       </c>
       <c r="B96" s="11" t="s">
@@ -9531,7 +9531,7 @@
       <c r="H96" s="1"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" s="36"/>
+      <c r="A97" s="45"/>
       <c r="B97" s="12"/>
       <c r="C97" s="12" t="s">
         <v>65</v>
@@ -9542,7 +9542,7 @@
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A98" s="36"/>
+      <c r="A98" s="45"/>
       <c r="B98" s="12"/>
       <c r="C98" s="12" t="s">
         <v>53</v>
@@ -9553,7 +9553,7 @@
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A99" s="36"/>
+      <c r="A99" s="45"/>
       <c r="B99" s="12"/>
       <c r="C99" s="12" t="s">
         <v>249</v>
@@ -9564,7 +9564,7 @@
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A100" s="36"/>
+      <c r="A100" s="45"/>
       <c r="B100" s="12"/>
       <c r="C100" s="12" t="s">
         <v>248</v>
@@ -9575,7 +9575,7 @@
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A101" s="36"/>
+      <c r="A101" s="45"/>
       <c r="B101" s="12"/>
       <c r="C101" s="12" t="s">
         <v>67</v>
@@ -9586,7 +9586,7 @@
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" s="36"/>
+      <c r="A102" s="45"/>
       <c r="B102" s="12"/>
       <c r="C102" s="12" t="s">
         <v>68</v>
@@ -9597,7 +9597,7 @@
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A103" s="36"/>
+      <c r="A103" s="45"/>
       <c r="B103" s="12"/>
       <c r="C103" s="12" t="s">
         <v>97</v>
@@ -9608,7 +9608,7 @@
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A104" s="36"/>
+      <c r="A104" s="45"/>
       <c r="B104" s="12"/>
       <c r="C104" s="22" t="s">
         <v>236</v>
@@ -9620,7 +9620,7 @@
       <c r="E104" s="12"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A105" s="36"/>
+      <c r="A105" s="45"/>
       <c r="D105">
         <f>-SUM(D96:D104)</f>
         <v>0</v>
@@ -9631,7 +9631,7 @@
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A106" s="36"/>
+      <c r="A106" s="45"/>
       <c r="B106" s="15" t="s">
         <v>63</v>
       </c>
@@ -9644,7 +9644,7 @@
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A107" s="36"/>
+      <c r="A107" s="45"/>
       <c r="B107" s="13"/>
       <c r="C107" s="13" t="s">
         <v>65</v>
@@ -9655,7 +9655,7 @@
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A108" s="36"/>
+      <c r="A108" s="45"/>
       <c r="B108" s="13"/>
       <c r="C108" s="13" t="s">
         <v>53</v>
@@ -9666,7 +9666,7 @@
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A109" s="36"/>
+      <c r="A109" s="45"/>
       <c r="B109" s="13"/>
       <c r="C109" s="13" t="s">
         <v>66</v>
@@ -9677,7 +9677,7 @@
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A110" s="36"/>
+      <c r="A110" s="45"/>
       <c r="B110" s="13"/>
       <c r="C110" s="13" t="s">
         <v>52</v>
@@ -9688,7 +9688,7 @@
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" s="36"/>
+      <c r="A111" s="45"/>
       <c r="B111" s="13"/>
       <c r="C111" s="13" t="s">
         <v>67</v>
@@ -9699,7 +9699,7 @@
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A112" s="36"/>
+      <c r="A112" s="45"/>
       <c r="B112" s="13"/>
       <c r="C112" s="13" t="s">
         <v>68</v>
@@ -9710,7 +9710,7 @@
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A113" s="36"/>
+      <c r="A113" s="45"/>
       <c r="B113" s="13"/>
       <c r="C113" s="13" t="s">
         <v>97</v>
@@ -9721,7 +9721,7 @@
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" s="36"/>
+      <c r="A114" s="45"/>
       <c r="B114" s="13"/>
       <c r="C114" s="22" t="s">
         <v>236</v>
@@ -9733,7 +9733,7 @@
       <c r="E114" s="13"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="36"/>
+      <c r="A115" s="45"/>
       <c r="D115">
         <f>-SUM(D106:D114)</f>
         <v>0</v>
@@ -9744,7 +9744,7 @@
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="36"/>
+      <c r="A116" s="45"/>
       <c r="B116" s="16" t="s">
         <v>63</v>
       </c>
@@ -9757,7 +9757,7 @@
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" s="36"/>
+      <c r="A117" s="45"/>
       <c r="B117" s="14"/>
       <c r="C117" s="14" t="s">
         <v>65</v>
@@ -9768,7 +9768,7 @@
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A118" s="36"/>
+      <c r="A118" s="45"/>
       <c r="B118" s="14"/>
       <c r="C118" s="14" t="s">
         <v>53</v>
@@ -9779,7 +9779,7 @@
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="36"/>
+      <c r="A119" s="45"/>
       <c r="B119" s="14"/>
       <c r="C119" s="14" t="s">
         <v>66</v>
@@ -9790,7 +9790,7 @@
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A120" s="36"/>
+      <c r="A120" s="45"/>
       <c r="B120" s="14"/>
       <c r="C120" s="14" t="s">
         <v>52</v>
@@ -9801,7 +9801,7 @@
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A121" s="36"/>
+      <c r="A121" s="45"/>
       <c r="B121" s="14"/>
       <c r="C121" s="14" t="s">
         <v>67</v>
@@ -9812,7 +9812,7 @@
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A122" s="36"/>
+      <c r="A122" s="45"/>
       <c r="B122" s="14"/>
       <c r="C122" s="14" t="s">
         <v>68</v>
@@ -9823,7 +9823,7 @@
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A123" s="36"/>
+      <c r="A123" s="45"/>
       <c r="B123" s="14"/>
       <c r="C123" s="14" t="s">
         <v>97</v>
@@ -9834,7 +9834,7 @@
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A124" s="36"/>
+      <c r="A124" s="45"/>
       <c r="B124" s="14"/>
       <c r="C124" s="22" t="s">
         <v>236</v>
@@ -9846,7 +9846,7 @@
       <c r="E124" s="14"/>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A125" s="36"/>
+      <c r="A125" s="45"/>
       <c r="D125">
         <f>-SUM(D116:D124)</f>
         <v>0</v>
@@ -11044,12 +11044,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="46" t="s">
         <v>253</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>

</xml_diff>